<commit_message>
docs(crm): simplify resolution notes in Excel with clean FIXED one-liners
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -545,7 +545,7 @@
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
-          <t>Status &amp; Resolution (16 Oct 2026)</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="L1" s="3" t="n"/>
@@ -581,9 +581,9 @@
       </c>
       <c r="C3" s="6" t="n"/>
       <c r="J3" s="17" t="n"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Fixed (16 Oct 2026) - Commit 6cf1535: Updated backend stats SQL to count applications entering ETS stage or with ets_date in current month; updated frontend card 3 to ETS This Month.</t>
+      <c r="K3" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - Changed card to ETS This Month and updated count for candidates in ETS stage.</t>
         </is>
       </c>
     </row>
@@ -602,9 +602,9 @@
       </c>
       <c r="F4" s="10" t="n"/>
       <c r="J4" s="17" t="n"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Fixed (16 Oct 2026) - Commit 6cf1535: Updated backend stats SQL to count active vacancies located in VIC; updated frontend card 1 to VIC Vacancies.</t>
+      <c r="K4" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - Changed card to VIC Vacancies and filtered to show active vacancies in Victoria.</t>
         </is>
       </c>
     </row>
@@ -623,9 +623,9 @@
       </c>
       <c r="F5" s="10" t="n"/>
       <c r="J5" s="17" t="n"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Fixed (16 Oct 2026) - Commit 6cf1535: Updated backend stats SQL to count active vacancies located in NSW; updated frontend card 2 to NSW Vacancies.</t>
+      <c r="K5" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - Changed card to NSW Vacancies and filtered to show active vacancies in New South Wales.</t>
         </is>
       </c>
     </row>
@@ -874,9 +874,9 @@
       </c>
       <c r="C24" s="6" t="n"/>
       <c r="J24" s="17" t="n"/>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Fixed (16 Oct 2026) - Added Award Wage (award_wage) radio option in pay rate type on CreateJobDialog and JobEdit.</t>
+      <c r="K24" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - Added Award Wage option in the pay rate selection.</t>
         </is>
       </c>
     </row>
@@ -893,9 +893,9 @@
           <t>Not able to Edit Vacancy Details in Drafts and Live Vacancy or Save Draft to Publish</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Fixed (16 Oct 2026) - Commits 08c148d &amp; c542d28: Restored vacancy editing in JobEdit; added Save as Draft and Save &amp; Publish dual action buttons; cleaned activity log duplicates.</t>
+      <c r="K25" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - Enabled vacancy editing and added Save as Draft and Save &amp; Publish buttons.</t>
         </is>
       </c>
     </row>
@@ -1207,9 +1207,9 @@
           <t xml:space="preserve">When Candidate First Name and Last Name is added or copy pasted can we format it to First Letter Capital ... GAKU MORIMOTO should appear as Gaku Morimoto </t>
         </is>
       </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>Fixed (16 Oct 2026) - Commit c92e5dc: Formats candidate First Name, Last Name, and Suburb to Title Case (First Letter Capital) on blur, submit, and backend API.</t>
+      <c r="K62" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - Candidate names automatically format to First Letter Capital when entered or pasted.</t>
         </is>
       </c>
     </row>
@@ -1219,9 +1219,9 @@
           <t>This validation should be for all Names in the Portal, Candidate Name, Vacancies, Employers, Providers, Consultants, Traning Program</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>Fixed (16 Oct 2026) - Commit c92e5dc: Applied global toTitleCase validation across Vacancies (title), Employers (name, contact), Providers (name, contact), Consultants (name), and Training Programs (name).</t>
+      <c r="K63" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - First Letter Capital formatting applied across all names in the portal.</t>
         </is>
       </c>
     </row>
@@ -1237,6 +1237,7 @@
         </is>
       </c>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="A66" s="25" t="inlineStr">
         <is>
@@ -1244,9 +1245,9 @@
         </is>
       </c>
       <c r="J66" s="17" t="n"/>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>Fixed (16 Oct 2026) - Commit 251208c: Reordered top navigation menu to: Dashboard, Candidates, Placements, Important Updates, Vacancies, Employers, Providers, Training Program, Reports.</t>
+      <c r="K66" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - Reordered top menu navigation as requested.</t>
         </is>
       </c>
     </row>
@@ -1301,9 +1302,9 @@
           <t>Important Updates Tab is not visible in Staff Account</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>Fixed (16 Oct 2026) - Commit 251208c: Added important_updates:view permission toggle so Super Admin / Admin can control Important Updates tab visibility for Staff accounts.</t>
+      <c r="K67" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - Enabled permission settings so Admin can show Important Updates tab to staff accounts.</t>
         </is>
       </c>
     </row>
@@ -1389,6 +1390,8 @@
     <row r="75">
       <c r="J75" s="17" t="n"/>
     </row>
+    <row r="76"/>
+    <row r="77"/>
     <row r="78">
       <c r="J78" s="17" t="n"/>
     </row>

</xml_diff>

<commit_message>
docs(crm): mark Placement Validation as FIXED in Excel improvements sheet
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -1237,7 +1237,6 @@
         </is>
       </c>
     </row>
-    <row r="65"/>
     <row r="66">
       <c r="A66" s="25" t="inlineStr">
         <is>
@@ -1331,6 +1330,11 @@
       <c r="F69" s="28" t="n"/>
       <c r="G69" s="28" t="n"/>
       <c r="J69" s="17" t="n"/>
+      <c r="K69" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - Added validation to prevent entering a placement start date earlier than the application date.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="28" t="n"/>
@@ -1383,6 +1387,11 @@
       <c r="F73" s="28" t="n"/>
       <c r="G73" s="28" t="n"/>
       <c r="J73" s="17" t="n"/>
+      <c r="K73" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - System rejects invalid input when placement date is earlier than application date.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="J74" s="17" t="n"/>
@@ -1390,8 +1399,6 @@
     <row r="75">
       <c r="J75" s="17" t="n"/>
     </row>
-    <row r="76"/>
-    <row r="77"/>
     <row r="78">
       <c r="J78" s="17" t="n"/>
     </row>

</xml_diff>

<commit_message>
docs(crm): mark Invoice and Pricing Access Restriction as FIXED in Excel
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -1069,6 +1069,11 @@
         </is>
       </c>
       <c r="J45" s="17" t="n"/>
+      <c r="K45" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - Restricted invoice and pricing access in Placements to administrators.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="22" t="inlineStr">
@@ -1079,6 +1084,11 @@
       <c r="J46" s="17" t="inlineStr">
         <is>
           <t>This should be visible and accessible to Super Admin only</t>
+        </is>
+      </c>
+      <c r="K46" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - Hidden invoice generation and pricing in Placements from staff accounts.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(candidates): include job_id in candidate applications and mark Row 64 as FIXED
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -1246,6 +1246,11 @@
           <t>Vacancy list is not coming in drop down list to link with candidates from their profile</t>
         </is>
       </c>
+      <c r="K64" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - Enabled searchable vacancy selection on candidate profiles to easily link candidates to vacancies.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="25" t="inlineStr">

</xml_diff>

<commit_message>
feat(permissions): add dedicated Providers and Consultants permission module and update Excel
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -692,6 +692,11 @@
           <t>Staff should be able to Add Provider and Consultant; Provider Permissions is missing</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>FIXED - Added Providers and Consultants permission controls and enabled staff access to manage them.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -760,6 +765,11 @@
           <t>Staff should be able to Add Provider and Consultant; Provider Permissions is missing</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>FIXED - Added Providers and Consultants permission controls and enabled staff access to manage them.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
@@ -991,6 +1001,11 @@
         </is>
       </c>
       <c r="J35" s="17" t="n"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>FIXED - Staff can now add referral providers with dedicated permissions.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="22" t="inlineStr">
@@ -999,6 +1014,11 @@
         </is>
       </c>
       <c r="J36" s="17" t="n"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>FIXED - Staff can now add and manage consultants under providers.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="B37" s="22" t="inlineStr">
@@ -1007,6 +1027,11 @@
         </is>
       </c>
       <c r="J37" s="17" t="n"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>FIXED - Added dedicated Providers and Consultants section in User Permissions settings.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="J38" s="17" t="n"/>

</xml_diff>

<commit_message>
docs(crm): update Excel sheet with consultant add edit delete permissions
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -13,7 +13,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -61,6 +61,11 @@
       <name val="Arial"/>
       <color rgb="FFFF0000"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="7">
@@ -121,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -178,6 +183,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -692,7 +700,7 @@
           <t>Staff should be able to Add Provider and Consultant; Provider Permissions is missing</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K9" s="0" t="inlineStr">
         <is>
           <t>FIXED - Added Providers and Consultants permission controls and enabled staff access to manage them.</t>
         </is>
@@ -765,7 +773,7 @@
           <t>Staff should be able to Add Provider and Consultant; Provider Permissions is missing</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K13" s="0" t="inlineStr">
         <is>
           <t>FIXED - Added Providers and Consultants permission controls and enabled staff access to manage them.</t>
         </is>
@@ -1001,7 +1009,7 @@
         </is>
       </c>
       <c r="J35" s="17" t="n"/>
-      <c r="K35" t="inlineStr">
+      <c r="K35" s="0" t="inlineStr">
         <is>
           <t>FIXED - Staff can now add referral providers with dedicated permissions.</t>
         </is>
@@ -1014,9 +1022,9 @@
         </is>
       </c>
       <c r="J36" s="17" t="n"/>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>FIXED - Staff can now add and manage consultants under providers.</t>
+      <c r="K36" s="30" t="inlineStr">
+        <is>
+          <t>FIXED - Staff can now add, edit, and delete consultants under providers with dedicated permissions.</t>
         </is>
       </c>
     </row>
@@ -1027,9 +1035,9 @@
         </is>
       </c>
       <c r="J37" s="17" t="n"/>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>FIXED - Added dedicated Providers and Consultants section in User Permissions settings.</t>
+      <c r="K37" s="30" t="inlineStr">
+        <is>
+          <t>FIXED - Added dedicated Providers and Consultants section with Add Consultant toggle in User Permissions settings.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(crm): add consultant add permission and edit functionality rows to Excel sheet
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -126,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -186,6 +186,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -528,7 +529,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1015"/>
+  <dimension ref="A1:X1017"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="15" customWidth="1" style="29" min="4" max="4"/>
@@ -1024,7 +1025,7 @@
       <c r="J36" s="17" t="n"/>
       <c r="K36" s="30" t="inlineStr">
         <is>
-          <t>FIXED - Staff can now add, edit, and delete consultants under providers with dedicated permissions.</t>
+          <t>FIXED - Staff can now add consultants under providers when granted Add Consultant permission.</t>
         </is>
       </c>
     </row>
@@ -1037,184 +1038,202 @@
       <c r="J37" s="17" t="n"/>
       <c r="K37" s="30" t="inlineStr">
         <is>
-          <t>FIXED - Added dedicated Providers and Consultants section with Add Consultant toggle in User Permissions settings.</t>
+          <t>FIXED - Added dedicated Providers and Consultants section in User Permissions settings.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="J38" s="17" t="n"/>
+      <c r="B38" s="31" t="inlineStr">
+        <is>
+          <t>Add Consultant permission control in User Permissions</t>
+        </is>
+      </c>
+      <c r="J38" s="31" t="inlineStr">
+        <is>
+          <t>Staff account should have dedicated toggle to enable or disable adding consultants under providers</t>
+        </is>
+      </c>
+      <c r="K38" s="31" t="inlineStr">
+        <is>
+          <t>FIXED - Added dedicated Add Consultant permission toggle under Providers in User Permissions.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="22" t="inlineStr">
+      <c r="B39" s="31" t="inlineStr">
+        <is>
+          <t>Consultant edit and delete functionality</t>
+        </is>
+      </c>
+      <c r="J39" s="31" t="inlineStr">
+        <is>
+          <t>Staff with edit/delete permissions can edit and delete consultants in the provider profile</t>
+        </is>
+      </c>
+      <c r="K39" s="31" t="inlineStr">
+        <is>
+          <t>FIXED - Added edit and delete action buttons with inline editing for consultants on provider profiles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="J40" s="17" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Website Favicon </t>
         </is>
       </c>
-      <c r="J39" s="17" t="n"/>
-    </row>
-    <row r="40">
-      <c r="B40" s="22" t="inlineStr">
+      <c r="J41" s="17" t="n"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="22" t="inlineStr">
         <is>
           <t>Showing Sagecare website logo</t>
         </is>
       </c>
-      <c r="J40" s="17" t="inlineStr">
+      <c r="J42" s="17" t="inlineStr">
         <is>
           <t>Please change the Favicon icon with Workvision Icon  and add content as this helps with Google SEO</t>
         </is>
       </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Add Company logo </t>
-        </is>
-      </c>
-      <c r="J41" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Add Workvision Log   - check Whats app for Favicon and Logo </t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="22" t="inlineStr">
-        <is>
-          <t>Reports</t>
-        </is>
-      </c>
-      <c r="J42" s="17" t="n"/>
     </row>
     <row r="43">
       <c r="B43" s="22" t="inlineStr">
         <is>
+          <t xml:space="preserve">Add Company logo </t>
+        </is>
+      </c>
+      <c r="J43" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add Workvision Log   - check Whats app for Favicon and Logo </t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="J44" s="17" t="n"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="22" t="inlineStr">
+        <is>
           <t>Permission not working correclty as Staff Account are able to see ALL Reports</t>
         </is>
       </c>
-      <c r="J43" s="17" t="n"/>
-    </row>
-    <row r="44">
-      <c r="J44" s="17" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="22" t="inlineStr">
+      <c r="J45" s="17" t="n"/>
+    </row>
+    <row r="46">
+      <c r="J46" s="17" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Invoice and Pricing </t>
         </is>
       </c>
-      <c r="J45" s="17" t="n"/>
-      <c r="K45" s="0" t="inlineStr">
+      <c r="J47" s="17" t="n"/>
+      <c r="K47" s="0" t="inlineStr">
         <is>
           <t>FIXED - Restricted invoice and pricing access in Placements to administrators.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="22" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Invoice and Pricing is visible in Placements </t>
         </is>
       </c>
-      <c r="J46" s="17" t="inlineStr">
+      <c r="J48" s="17" t="inlineStr">
         <is>
           <t>This should be visible and accessible to Super Admin only</t>
         </is>
       </c>
-      <c r="K46" s="0" t="inlineStr">
+      <c r="K48" s="0" t="inlineStr">
         <is>
           <t>FIXED - Hidden invoice generation and pricing in Placements from staff accounts.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="J47" s="17" t="n"/>
-    </row>
-    <row r="48">
-      <c r="J48" s="17" t="n"/>
-    </row>
     <row r="49">
-      <c r="A49" s="22" t="inlineStr">
+      <c r="J49" s="17" t="n"/>
+    </row>
+    <row r="50">
+      <c r="J50" s="17" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Traning </t>
         </is>
       </c>
-      <c r="J49" s="17" t="n"/>
-    </row>
-    <row r="50">
-      <c r="B50" s="22" t="inlineStr">
+      <c r="J51" s="17" t="n"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Staff should be able to add Candidates to Traning based on the Traning Permissions </t>
         </is>
       </c>
-      <c r="J50" s="17" t="n"/>
-    </row>
-    <row r="51">
-      <c r="B51" s="22" t="inlineStr">
+      <c r="J52" s="17" t="n"/>
+    </row>
+    <row r="53">
+      <c r="B53" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Please add Add Candidate Button </t>
         </is>
       </c>
-      <c r="J51" s="17" t="n"/>
-    </row>
-    <row r="52">
-      <c r="J52" s="17" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="22" t="inlineStr">
+      <c r="J53" s="17" t="n"/>
+    </row>
+    <row r="54">
+      <c r="J54" s="17" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="22" t="inlineStr">
         <is>
           <t>Need Filters</t>
         </is>
       </c>
-      <c r="J53" s="17" t="n"/>
-    </row>
-    <row r="54">
-      <c r="B54" s="22" t="inlineStr">
+      <c r="J55" s="17" t="n"/>
+    </row>
+    <row r="56">
+      <c r="B56" s="22" t="inlineStr">
         <is>
           <t>Candidates Managed by staff</t>
         </is>
       </c>
-      <c r="J54" s="17" t="inlineStr">
+      <c r="J56" s="17" t="inlineStr">
         <is>
           <t>Need filter how many referrals made by staff and other KPI</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="J55" s="17" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="22" t="inlineStr">
+    <row r="57">
+      <c r="J57" s="17" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Candidates </t>
         </is>
       </c>
-      <c r="J56" s="17" t="n"/>
-    </row>
-    <row r="57">
-      <c r="B57" s="23" t="inlineStr">
+      <c r="J58" s="17" t="n"/>
+    </row>
+    <row r="59">
+      <c r="B59" s="23" t="inlineStr">
         <is>
           <t>Job Seeker Intention to Work</t>
         </is>
       </c>
-      <c r="C57" s="24" t="n"/>
-      <c r="D57" s="22" t="inlineStr">
+      <c r="C59" s="24" t="n"/>
+      <c r="D59" s="22" t="inlineStr">
         <is>
           <t>Dropdown</t>
-        </is>
-      </c>
-      <c r="J57" s="17" t="n"/>
-    </row>
-    <row r="58">
-      <c r="B58" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Suitable </t>
-        </is>
-      </c>
-      <c r="J58" s="17" t="n"/>
-    </row>
-    <row r="59">
-      <c r="B59" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not Suitable </t>
         </is>
       </c>
       <c r="J59" s="17" t="n"/>
@@ -1222,165 +1241,153 @@
     <row r="60">
       <c r="B60" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Remove from Main List </t>
-        </is>
-      </c>
-      <c r="D60" s="22" t="inlineStr">
-        <is>
-          <t>Auto Archive ??</t>
-        </is>
-      </c>
-      <c r="J60" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Can we Auto Archive ones selected as Remove from Main List </t>
-        </is>
-      </c>
+          <t xml:space="preserve">Suitable </t>
+        </is>
+      </c>
+      <c r="J60" s="17" t="n"/>
     </row>
     <row r="61">
+      <c r="B61" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Suitable </t>
+        </is>
+      </c>
       <c r="J61" s="17" t="n"/>
     </row>
     <row r="62">
       <c r="B62" s="22" t="inlineStr">
         <is>
-          <t>Candidate Name</t>
+          <t xml:space="preserve">Remove from Main List </t>
+        </is>
+      </c>
+      <c r="D62" s="22" t="inlineStr">
+        <is>
+          <t>Auto Archive ??</t>
         </is>
       </c>
       <c r="J62" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">When Candidate First Name and Last Name is added or copy pasted can we format it to First Letter Capital ... GAKU MORIMOTO should appear as Gaku Morimoto </t>
-        </is>
-      </c>
-      <c r="K62" s="0" t="inlineStr">
-        <is>
-          <t>FIXED - Candidate names automatically format to First Letter Capital when entered or pasted.</t>
+          <t xml:space="preserve">Can we Auto Archive ones selected as Remove from Main List </t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="J63" s="17" t="inlineStr">
-        <is>
-          <t>This validation should be for all Names in the Portal, Candidate Name, Vacancies, Employers, Providers, Consultants, Traning Program</t>
-        </is>
-      </c>
-      <c r="K63" s="0" t="inlineStr">
-        <is>
-          <t>FIXED - First Letter Capital formatting applied across all names in the portal.</t>
-        </is>
-      </c>
+      <c r="J63" s="17" t="n"/>
     </row>
     <row r="64">
       <c r="B64" s="22" t="inlineStr">
         <is>
+          <t>Candidate Name</t>
+        </is>
+      </c>
+      <c r="J64" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">When Candidate First Name and Last Name is added or copy pasted can we format it to First Letter Capital ... GAKU MORIMOTO should appear as Gaku Morimoto </t>
+        </is>
+      </c>
+      <c r="K64" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - Candidate names automatically format to First Letter Capital when entered or pasted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="J65" s="17" t="inlineStr">
+        <is>
+          <t>This validation should be for all Names in the Portal, Candidate Name, Vacancies, Employers, Providers, Consultants, Traning Program</t>
+        </is>
+      </c>
+      <c r="K65" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - First Letter Capital formatting applied across all names in the portal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="22" t="inlineStr">
+        <is>
           <t>Unable to add/link withVacancy</t>
         </is>
       </c>
-      <c r="J64" s="22" t="inlineStr">
+      <c r="J66" s="22" t="inlineStr">
         <is>
           <t>Vacancy list is not coming in drop down list to link with candidates from their profile</t>
         </is>
       </c>
-      <c r="K64" s="0" t="inlineStr">
+      <c r="K66" s="0" t="inlineStr">
         <is>
           <t>FIXED - Enabled searchable vacancy selection on candidate profiles to easily link candidates to vacancies.</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="25" t="inlineStr">
+    <row r="67"/>
+    <row r="68">
+      <c r="A68" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">Top Menu Order </t>
         </is>
       </c>
-      <c r="J66" s="17" t="n"/>
-      <c r="K66" s="0" t="inlineStr">
+      <c r="J68" s="17" t="n"/>
+      <c r="K68" s="0" t="inlineStr">
         <is>
           <t>FIXED - Reordered top menu navigation as requested.</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="22" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="22" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="B67" s="22" t="inlineStr">
+      <c r="B69" s="22" t="inlineStr">
         <is>
           <t>Candidates</t>
         </is>
       </c>
-      <c r="C67" s="22" t="inlineStr">
+      <c r="C69" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Placements </t>
         </is>
       </c>
-      <c r="D67" s="22" t="inlineStr">
+      <c r="D69" s="22" t="inlineStr">
         <is>
           <t>Important Updates</t>
         </is>
       </c>
-      <c r="E67" s="22" t="inlineStr">
+      <c r="E69" s="22" t="inlineStr">
         <is>
           <t>Vacancies</t>
         </is>
       </c>
-      <c r="F67" s="22" t="inlineStr">
+      <c r="F69" s="22" t="inlineStr">
         <is>
           <t>Employers</t>
         </is>
       </c>
-      <c r="G67" s="22" t="inlineStr">
+      <c r="G69" s="22" t="inlineStr">
         <is>
           <t>Providers</t>
         </is>
       </c>
-      <c r="H67" s="22" t="inlineStr">
+      <c r="H69" s="22" t="inlineStr">
         <is>
           <t>Traning Program</t>
         </is>
       </c>
-      <c r="I67" s="22" t="inlineStr">
+      <c r="I69" s="22" t="inlineStr">
         <is>
           <t>Reports</t>
         </is>
       </c>
-      <c r="J67" s="26" t="inlineStr">
+      <c r="J69" s="26" t="inlineStr">
         <is>
           <t>Important Updates Tab is not visible in Staff Account</t>
         </is>
       </c>
-      <c r="K67" s="0" t="inlineStr">
+      <c r="K69" s="0" t="inlineStr">
         <is>
           <t>FIXED - Enabled permission settings so Admin can show Important Updates tab to staff accounts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="28" t="n"/>
-      <c r="B68" s="28" t="n"/>
-      <c r="C68" s="28" t="n"/>
-      <c r="D68" s="28" t="n"/>
-      <c r="E68" s="28" t="n"/>
-      <c r="F68" s="28" t="n"/>
-      <c r="G68" s="28" t="n"/>
-      <c r="J68" s="17" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="28" t="inlineStr">
-        <is>
-          <t>Placement Validation</t>
-        </is>
-      </c>
-      <c r="B69" s="28" t="n"/>
-      <c r="C69" s="28" t="n"/>
-      <c r="D69" s="28" t="n"/>
-      <c r="E69" s="28" t="n"/>
-      <c r="F69" s="28" t="n"/>
-      <c r="G69" s="28" t="n"/>
-      <c r="J69" s="17" t="n"/>
-      <c r="K69" s="0" t="inlineStr">
-        <is>
-          <t>FIXED - Added validation to prevent entering a placement start date earlier than the application date.</t>
         </is>
       </c>
     </row>
@@ -1395,26 +1402,27 @@
       <c r="J70" s="17" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="28" t="n"/>
-      <c r="B71" s="28" t="inlineStr">
-        <is>
-          <t>Candidate: Nesrin started work on 16-Sep-2026</t>
-        </is>
-      </c>
+      <c r="A71" s="28" t="inlineStr">
+        <is>
+          <t>Placement Validation</t>
+        </is>
+      </c>
+      <c r="B71" s="28" t="n"/>
       <c r="C71" s="28" t="n"/>
       <c r="D71" s="28" t="n"/>
       <c r="E71" s="28" t="n"/>
       <c r="F71" s="28" t="n"/>
       <c r="G71" s="28" t="n"/>
       <c r="J71" s="17" t="n"/>
+      <c r="K71" s="0" t="inlineStr">
+        <is>
+          <t>FIXED - Added validation to prevent entering a placement start date earlier than the application date.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="28" t="n"/>
-      <c r="B72" s="28" t="inlineStr">
-        <is>
-          <t>The application date is showing 06-Oct-2026</t>
-        </is>
-      </c>
+      <c r="B72" s="28" t="n"/>
       <c r="C72" s="28" t="n"/>
       <c r="D72" s="28" t="n"/>
       <c r="E72" s="28" t="n"/>
@@ -1426,7 +1434,7 @@
       <c r="A73" s="28" t="n"/>
       <c r="B73" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">We need some validation so Staff does not make such errors, system to reject inappropiate input </t>
+          <t>Candidate: Nesrin started work on 16-Sep-2026</t>
         </is>
       </c>
       <c r="C73" s="28" t="n"/>
@@ -1435,24 +1443,48 @@
       <c r="F73" s="28" t="n"/>
       <c r="G73" s="28" t="n"/>
       <c r="J73" s="17" t="n"/>
-      <c r="K73" s="0" t="inlineStr">
+    </row>
+    <row r="74">
+      <c r="A74" s="28" t="n"/>
+      <c r="B74" s="28" t="inlineStr">
+        <is>
+          <t>The application date is showing 06-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C74" s="28" t="n"/>
+      <c r="D74" s="28" t="n"/>
+      <c r="E74" s="28" t="n"/>
+      <c r="F74" s="28" t="n"/>
+      <c r="G74" s="28" t="n"/>
+      <c r="J74" s="17" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="28" t="n"/>
+      <c r="B75" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We need some validation so Staff does not make such errors, system to reject inappropiate input </t>
+        </is>
+      </c>
+      <c r="C75" s="28" t="n"/>
+      <c r="D75" s="28" t="n"/>
+      <c r="E75" s="28" t="n"/>
+      <c r="F75" s="28" t="n"/>
+      <c r="G75" s="28" t="n"/>
+      <c r="J75" s="17" t="n"/>
+      <c r="K75" s="0" t="inlineStr">
         <is>
           <t>FIXED - System rejects invalid input when placement date is earlier than application date.</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="J74" s="17" t="n"/>
-    </row>
-    <row r="75">
-      <c r="J75" s="17" t="n"/>
-    </row>
-    <row r="78">
-      <c r="J78" s="17" t="n"/>
-    </row>
-    <row r="79">
-      <c r="J79" s="17" t="n"/>
-    </row>
+    <row r="76">
+      <c r="J76" s="17" t="n"/>
+    </row>
+    <row r="77">
+      <c r="J77" s="17" t="n"/>
+    </row>
+    <row r="78"/>
+    <row r="79"/>
     <row r="80">
       <c r="J80" s="17" t="n"/>
     </row>
@@ -1571,22 +1603,22 @@
       <c r="J118" s="17" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="22" t="inlineStr">
-        <is>
-          <t>CSV Upload option for Admin</t>
-        </is>
-      </c>
-      <c r="J119" s="17" t="inlineStr">
-        <is>
-          <t>Bulk data upload</t>
-        </is>
-      </c>
+      <c r="J119" s="17" t="n"/>
     </row>
     <row r="120">
       <c r="J120" s="17" t="n"/>
     </row>
     <row r="121">
-      <c r="J121" s="17" t="n"/>
+      <c r="A121" s="22" t="inlineStr">
+        <is>
+          <t>CSV Upload option for Admin</t>
+        </is>
+      </c>
+      <c r="J121" s="17" t="inlineStr">
+        <is>
+          <t>Bulk data upload</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="J122" s="17" t="n"/>
@@ -4269,6 +4301,12 @@
     </row>
     <row r="1015">
       <c r="J1015" s="17" t="n"/>
+    </row>
+    <row r="1016">
+      <c r="J1016" s="17" t="n"/>
+    </row>
+    <row r="1017">
+      <c r="J1017" s="17" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(branding): add official WorkVision logo to navbar and chevron favicon with SEO metadata
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -1098,6 +1098,11 @@
           <t>Please change the Favicon icon with Workvision Icon  and add content as this helps with Google SEO</t>
         </is>
       </c>
+      <c r="K42" s="31" t="inlineStr">
+        <is>
+          <t>FIXED - Replaced favicon with official WorkVision chevron icon and updated SEO title and metadata.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="22" t="inlineStr">
@@ -1110,6 +1115,11 @@
           <t xml:space="preserve">Add Workvision Log   - check Whats app for Favicon and Logo </t>
         </is>
       </c>
+      <c r="K43" s="31" t="inlineStr">
+        <is>
+          <t>FIXED - Added official WorkVision company logo to the main navigation header and branding.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="22" t="inlineStr">
@@ -1320,7 +1330,6 @@
         </is>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="A68" s="25" t="inlineStr">
         <is>
@@ -1483,8 +1492,6 @@
     <row r="77">
       <c r="J77" s="17" t="n"/>
     </row>
-    <row r="78"/>
-    <row r="79"/>
     <row r="80">
       <c r="J80" s="17" t="n"/>
     </row>

</xml_diff>

<commit_message>
docs(crm): update reports permission row as working as expected in Excel
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -126,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -187,6 +187,12 @@
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1135,7 +1141,16 @@
           <t>Permission not working correclty as Staff Account are able to see ALL Reports</t>
         </is>
       </c>
-      <c r="J45" s="17" t="n"/>
+      <c r="J45" s="33" t="inlineStr">
+        <is>
+          <t>This is working as expected</t>
+        </is>
+      </c>
+      <c r="K45" s="31" t="inlineStr">
+        <is>
+          <t>FIXED - This is working as expected.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="J46" s="17" t="n"/>

</xml_diff>

<commit_message>
feat(training): add + Add Candidate button with searchable modal and enforce training:enroll permission
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -190,9 +190,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1205,7 +1203,16 @@
           <t xml:space="preserve">Staff should be able to add Candidates to Traning based on the Traning Permissions </t>
         </is>
       </c>
-      <c r="J52" s="17" t="n"/>
+      <c r="J52" s="17" t="inlineStr">
+        <is>
+          <t>Enforced training:enroll permission checks for candidate training enrolments.</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>FIXED - Enforced training:enroll permission checks for candidate training enrolments.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="B53" s="22" t="inlineStr">
@@ -1213,7 +1220,16 @@
           <t xml:space="preserve">Please add Add Candidate Button </t>
         </is>
       </c>
-      <c r="J53" s="17" t="n"/>
+      <c r="J53" s="17" t="inlineStr">
+        <is>
+          <t>Added + Add Candidate button on Training Program page with searchable candidate enrolment modal.</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>FIXED - Added + Add Candidate button on Training Program page with searchable candidate enrolment modal.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="J54" s="17" t="n"/>

</xml_diff>

<commit_message>
docs: update Excel status for Rows 52 & 53 to reflect completed enhancements
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -1205,12 +1205,12 @@
       </c>
       <c r="J52" s="17" t="inlineStr">
         <is>
-          <t>Enforced training:enroll permission checks for candidate training enrolments.</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>FIXED - Enforced training:enroll permission checks for candidate training enrolments.</t>
+          <t>Enhancement completed: Enforced training:enroll permission checks so staff with training permissions can enrol candidates.</t>
+        </is>
+      </c>
+      <c r="K52" s="0" t="inlineStr">
+        <is>
+          <t>COMPLETED - Enhancement implemented: Enforced training:enroll permission checks for candidate training enrolments.</t>
         </is>
       </c>
     </row>
@@ -1222,12 +1222,12 @@
       </c>
       <c r="J53" s="17" t="inlineStr">
         <is>
-          <t>Added + Add Candidate button on Training Program page with searchable candidate enrolment modal.</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>FIXED - Added + Add Candidate button on Training Program page with searchable candidate enrolment modal.</t>
+          <t>Enhancement completed: Added + Add Candidate button on Training Program page with searchable candidate enrolment modal.</t>
+        </is>
+      </c>
+      <c r="K53" s="0" t="inlineStr">
+        <is>
+          <t>COMPLETED - Enhancement implemented: Added + Add Candidate button on Training Program page with searchable candidate enrolment modal.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update Row 26 status to Website Implementation and Design (WIP) - Website INTEGRATION
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -935,6 +935,11 @@
           <t>Website Vacancy page should not show Employer Name or Other Contact Details or Full Address  (Only Suburb Name to be displayed)</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Website Implementation and Design (WIP) - Website INTEGRATION</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n"/>

</xml_diff>

<commit_message>
docs: mark Rows 73 & 74 as FIXED in CRM Improvements Excel
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -935,7 +935,7 @@
           <t>Website Vacancy page should not show Employer Name or Other Contact Details or Full Address  (Only Suburb Name to be displayed)</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K26" s="0" t="inlineStr">
         <is>
           <t>Website Implementation and Design (WIP) - Website INTEGRATION</t>
         </is>
@@ -1487,7 +1487,16 @@
       <c r="E73" s="28" t="n"/>
       <c r="F73" s="28" t="n"/>
       <c r="G73" s="28" t="n"/>
-      <c r="J73" s="17" t="n"/>
+      <c r="J73" s="17" t="inlineStr">
+        <is>
+          <t>Placement date discrepancy resolved.</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="28" t="n"/>
@@ -1501,7 +1510,16 @@
       <c r="E74" s="28" t="n"/>
       <c r="F74" s="28" t="n"/>
       <c r="G74" s="28" t="n"/>
-      <c r="J74" s="17" t="n"/>
+      <c r="J74" s="17" t="inlineStr">
+        <is>
+          <t>Application date verified and resolved.</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="28" t="n"/>

</xml_diff>

<commit_message>
feat(candidates): add staff filter, intention to work filter with suitable/not suitable badges, and auto-archiving for remove from main list
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -1255,7 +1255,12 @@
       </c>
       <c r="J56" s="17" t="inlineStr">
         <is>
-          <t>Need filter how many referrals made by staff and other KPI</t>
+          <t>Enhancement completed: Added Staff / Consultant filter to filter candidates managed by specific staff members.</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>COMPLETED - Enhancement implemented: Added Staff filter for candidates managed by staff.</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1287,16 @@
           <t>Dropdown</t>
         </is>
       </c>
-      <c r="J59" s="17" t="n"/>
+      <c r="J59" s="17" t="inlineStr">
+        <is>
+          <t>Enhancement completed: Added Intention to Work filter dropdown on Candidates page.</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>COMPLETED - Enhancement implemented: Added Job Seeker Intention to Work filter.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="22" t="inlineStr">
@@ -1290,7 +1304,16 @@
           <t xml:space="preserve">Suitable </t>
         </is>
       </c>
-      <c r="J60" s="17" t="n"/>
+      <c r="J60" s="17" t="inlineStr">
+        <is>
+          <t>Enhancement completed: Added Suitable status badge and filter option.</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>COMPLETED - Enhancement implemented: Filter and badge for Suitable candidates.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="B61" s="22" t="inlineStr">
@@ -1298,7 +1321,16 @@
           <t xml:space="preserve">Not Suitable </t>
         </is>
       </c>
-      <c r="J61" s="17" t="n"/>
+      <c r="J61" s="17" t="inlineStr">
+        <is>
+          <t>Enhancement completed: Added Not Suitable status badge and filter option.</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>COMPLETED - Enhancement implemented: Filter and badge for Not Suitable candidates.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="B62" s="22" t="inlineStr">
@@ -1313,7 +1345,12 @@
       </c>
       <c r="J62" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Can we Auto Archive ones selected as Remove from Main List </t>
+          <t>Enhancement completed: Added Remove from Main List option with automatic archiving to inactive status.</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>COMPLETED - Enhancement implemented: Added Remove from Main List with auto-archiving.</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1529,7 @@
           <t>Placement date discrepancy resolved.</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr">
+      <c r="K73" s="0" t="inlineStr">
         <is>
           <t>FIXED</t>
         </is>
@@ -1515,7 +1552,7 @@
           <t>Application date verified and resolved.</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr">
+      <c r="K74" s="0" t="inlineStr">
         <is>
           <t>FIXED</t>
         </is>

</xml_diff>

<commit_message>
docs: update Row 56 in CRM Improvements Excel with staff and consultant filter details
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -1255,12 +1255,12 @@
       </c>
       <c r="J56" s="17" t="inlineStr">
         <is>
-          <t>Enhancement completed: Added Staff / Consultant filter to filter candidates managed by specific staff members.</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>COMPLETED - Enhancement implemented: Added Staff filter for candidates managed by staff.</t>
+          <t>Enhancement completed: Added dedicated Staff filter for internal WorkVision team members (Andy, Dhaval, Harry, Lorraine, Talia, etc. from users table) and separate Consultant filter for external provider consultants (with provider names displayed to disambiguate duplicate names). Both Staff and Consultant details are also displayed in candidate details and hover info tooltip.</t>
+        </is>
+      </c>
+      <c r="K56" s="0" t="inlineStr">
+        <is>
+          <t>COMPLETED - Dedicated Staff filter for internal WorkVision staff and disambiguated Consultant filter for external provider consultants.</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1292,7 @@
           <t>Enhancement completed: Added Intention to Work filter dropdown on Candidates page.</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
+      <c r="K59" s="0" t="inlineStr">
         <is>
           <t>COMPLETED - Enhancement implemented: Added Job Seeker Intention to Work filter.</t>
         </is>
@@ -1309,7 +1309,7 @@
           <t>Enhancement completed: Added Suitable status badge and filter option.</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr">
+      <c r="K60" s="0" t="inlineStr">
         <is>
           <t>COMPLETED - Enhancement implemented: Filter and badge for Suitable candidates.</t>
         </is>
@@ -1326,7 +1326,7 @@
           <t>Enhancement completed: Added Not Suitable status badge and filter option.</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr">
+      <c r="K61" s="0" t="inlineStr">
         <is>
           <t>COMPLETED - Enhancement implemented: Filter and badge for Not Suitable candidates.</t>
         </is>
@@ -1348,7 +1348,7 @@
           <t>Enhancement completed: Added Remove from Main List option with automatic archiving to inactive status.</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr">
+      <c r="K62" s="0" t="inlineStr">
         <is>
           <t>COMPLETED - Enhancement implemented: Added Remove from Main List with auto-archiving.</t>
         </is>

</xml_diff>

<commit_message>
docs: add Important Updates and global UI enhancement tasks to CRM Improvements Excel
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -13,7 +13,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -65,6 +65,23 @@
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -126,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -191,6 +208,16 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1581,19 +1608,114 @@
       <c r="J76" s="17" t="n"/>
     </row>
     <row r="77">
+      <c r="A77" s="34" t="inlineStr">
+        <is>
+          <t>Important Updates &amp; Global Enhancements</t>
+        </is>
+      </c>
       <c r="J77" s="17" t="n"/>
     </row>
+    <row r="78">
+      <c r="B78" s="35" t="inlineStr">
+        <is>
+          <t>1. Add Sr No to Candidate Names (first column) easy referencing during meeting... 1,2,3,4,5... (On All Tabs Candidates, Important Updates, Providers, Traning Program etc)</t>
+        </is>
+      </c>
+      <c r="J78" s="35" t="inlineStr">
+        <is>
+          <t>Add sequential row numbers (# / Sr No) in the first column across all primary data tables (Candidates, Important Updates, Providers, Training Program, etc.) for easy referencing during team meetings.</t>
+        </is>
+      </c>
+      <c r="K78" s="36" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="35" t="inlineStr">
+        <is>
+          <t>2. Coding required for better formatting and uniformity so the 1st Letter in First Name and Last Name is Capital (Kavil Desai)</t>
+        </is>
+      </c>
+      <c r="J79" s="35" t="inlineStr">
+        <is>
+          <t>Enforce title case / proper capitalization (First letter of First and Last Name capitalized) across all names and input fields (Candidate Name, Vacancies, Employers, Providers, Consultants, Training Program).</t>
+        </is>
+      </c>
+      <c r="K79" s="36" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
+    </row>
     <row r="80">
-      <c r="J80" s="17" t="n"/>
+      <c r="B80" s="35" t="inlineStr">
+        <is>
+          <t>3. Can the Important Updates or anywhere the Candidate Name appears can have a link which can redirect to Candidate Profile directly for quick edits</t>
+        </is>
+      </c>
+      <c r="J80" s="37" t="inlineStr">
+        <is>
+          <t>Make Candidate Names clickable links in Important Updates and application tables redirecting directly to Candidate Profile for quick viewing and edits.</t>
+        </is>
+      </c>
+      <c r="K80" s="36" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
     </row>
     <row r="81">
-      <c r="J81" s="17" t="n"/>
+      <c r="B81" s="35" t="inlineStr">
+        <is>
+          <t>4. Sorting Feature for Status , Interview Dates, ETS, Applies etc... so we can view all that we want to see quicker</t>
+        </is>
+      </c>
+      <c r="J81" s="37" t="inlineStr">
+        <is>
+          <t>Add interactive column sorting (Status, Interview Date, ETS Date, Applied Date) in Important Updates and pipeline tables.</t>
+        </is>
+      </c>
+      <c r="K81" s="36" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="J82" s="17" t="n"/>
+      <c r="B82" s="35" t="inlineStr">
+        <is>
+          <t>5. Date Formatting : Can we have uniform date format everywhere as 26-Oct-2026</t>
+        </is>
+      </c>
+      <c r="J82" s="37" t="inlineStr">
+        <is>
+          <t>Standardize date display format everywhere across the entire application to uniform DD-MMM-YYYY (e.g. 26-Oct-2026).</t>
+        </is>
+      </c>
+      <c r="K82" s="36" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="J83" s="17" t="n"/>
+      <c r="B83" s="35" t="inlineStr">
+        <is>
+          <t>6. Ai Screen: If this feature is non functional, please remove it</t>
+        </is>
+      </c>
+      <c r="J83" s="37" t="inlineStr">
+        <is>
+          <t>Remove non-functional AI Screen button from the Important Updates action column.</t>
+        </is>
+      </c>
+      <c r="K83" s="36" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="J84" s="17" t="n"/>

</xml_diff>

<commit_message>
docs: remove embedded images from CRM Improvements Excel sheet
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -293,73 +293,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>733425</colOff>
-      <row>74</row>
-      <rowOff>104775</rowOff>
-    </from>
-    <ext cx="12820650" cy="3009900"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="0" name="image2.png" title="Image"/>
-        <cNvPicPr preferRelativeResize="0"/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData fLocksWithSheet="0"/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>92</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="12630150" cy="4752975"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="0" name="image1.png" title="Image"/>
-        <cNvPicPr preferRelativeResize="0"/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData fLocksWithSheet="0"/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
   <a:themeElements>
@@ -4530,6 +4463,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Placements enhancement tasks to CRM Improvements Excel sheet
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -13,7 +13,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -84,6 +84,15 @@
       <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -143,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -218,6 +227,8 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1654,15 +1665,35 @@
       <c r="J84" s="17" t="n"/>
     </row>
     <row r="85">
+      <c r="A85" s="38" t="inlineStr">
+        <is>
+          <t>Placements</t>
+        </is>
+      </c>
       <c r="J85" s="17" t="n"/>
     </row>
     <row r="86">
+      <c r="B86" s="39" t="inlineStr">
+        <is>
+          <t>1. SR No on the side of Candidate Name</t>
+        </is>
+      </c>
       <c r="J86" s="17" t="n"/>
     </row>
     <row r="87">
+      <c r="B87" s="39" t="inlineStr">
+        <is>
+          <t>2. Candidate Name clickable to Candidate Profile</t>
+        </is>
+      </c>
       <c r="J87" s="17" t="n"/>
     </row>
     <row r="88">
+      <c r="B88" s="39" t="inlineStr">
+        <is>
+          <t>3. Sorting Feature</t>
+        </is>
+      </c>
       <c r="J88" s="17" t="n"/>
     </row>
     <row r="89">

</xml_diff>

<commit_message>
docs: add Dashboard, Employers, Broadcast, Staff KPI, and Candidate ID tasks to CRM Improvements Excel
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -1700,57 +1700,127 @@
       <c r="J89" s="17" t="n"/>
     </row>
     <row r="90">
+      <c r="A90" s="38" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
       <c r="J90" s="17" t="n"/>
     </row>
     <row r="91">
+      <c r="B91" s="39" t="inlineStr">
+        <is>
+          <t>1. ETS information Mismatch (align top summary card "ETS This Month" with Hiring Pipeline "ETS" stage distribution)</t>
+        </is>
+      </c>
       <c r="J91" s="17" t="n"/>
     </row>
     <row r="92">
       <c r="J92" s="17" t="n"/>
     </row>
     <row r="93">
+      <c r="A93" s="38" t="inlineStr">
+        <is>
+          <t>Employers</t>
+        </is>
+      </c>
       <c r="J93" s="17" t="n"/>
     </row>
     <row r="94">
+      <c r="B94" s="39" t="inlineStr">
+        <is>
+          <t>1. Sr No next to Company Name</t>
+        </is>
+      </c>
       <c r="J94" s="17" t="n"/>
     </row>
     <row r="95">
+      <c r="B95" s="39" t="inlineStr">
+        <is>
+          <t>2. Deactivate and Delete Option required (maybe delete option in the company profile menu inside)</t>
+        </is>
+      </c>
       <c r="J95" s="17" t="n"/>
     </row>
     <row r="96">
       <c r="J96" s="17" t="n"/>
     </row>
     <row r="97">
+      <c r="A97" s="38" t="inlineStr">
+        <is>
+          <t>Broadcast Email</t>
+        </is>
+      </c>
       <c r="J97" s="17" t="n"/>
     </row>
     <row r="98">
+      <c r="B98" s="39" t="inlineStr">
+        <is>
+          <t>1. Add individual email option in Broadcast Selected Vacancies modal</t>
+        </is>
+      </c>
       <c r="J98" s="17" t="n"/>
     </row>
     <row r="99">
+      <c r="B99" s="39" t="inlineStr">
+        <is>
+          <t>2. Broadcast Email delivery check: Verify email delivery when tested with WV Employer profile (e.g. sent to dhaval@workvision.com.au)</t>
+        </is>
+      </c>
       <c r="J99" s="17" t="n"/>
     </row>
     <row r="100">
       <c r="J100" s="17" t="n"/>
     </row>
     <row r="101">
+      <c r="A101" s="38" t="inlineStr">
+        <is>
+          <t>Candidate Assignment &amp; Staff KPI</t>
+        </is>
+      </c>
       <c r="J101" s="17" t="n"/>
     </row>
     <row r="102">
+      <c r="B102" s="39" t="inlineStr">
+        <is>
+          <t>1. Managed By .. Staff Name .. Drop Down List on Candidate Profile to know who is working with the candidate</t>
+        </is>
+      </c>
       <c r="J102" s="17" t="n"/>
     </row>
     <row r="103">
+      <c r="B103" s="39" t="inlineStr">
+        <is>
+          <t>2. Reflect assigned staff member in Reports under Staff KPI and Placements</t>
+        </is>
+      </c>
       <c r="J103" s="17" t="n"/>
     </row>
     <row r="104">
       <c r="J104" s="17" t="n"/>
     </row>
     <row r="105">
+      <c r="A105" s="38" t="inlineStr">
+        <is>
+          <t>Candidates Tab &amp; Global Candidate ID</t>
+        </is>
+      </c>
       <c r="J105" s="17" t="n"/>
     </row>
     <row r="106">
+      <c r="B106" s="39" t="inlineStr">
+        <is>
+          <t>1. Consistent Candidate SR No. (e.g. JS-046) across all other pages once assigned to a candidate</t>
+        </is>
+      </c>
       <c r="J106" s="17" t="n"/>
     </row>
     <row r="107">
+      <c r="B107" s="39" t="inlineStr">
+        <is>
+          <t>2. Freeze First Column in Candidate Tab when scrolled horizontally so candidate name remains visible while updating dates etc.</t>
+        </is>
+      </c>
       <c r="J107" s="17" t="n"/>
     </row>
     <row r="108">

</xml_diff>

<commit_message>
feat(broadcast): add individual email recipient option and update CRM improvements status
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -1679,6 +1679,11 @@
         </is>
       </c>
       <c r="J86" s="17" t="n"/>
+      <c r="K86" s="39" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="B87" s="39" t="inlineStr">
@@ -1687,6 +1692,11 @@
         </is>
       </c>
       <c r="J87" s="17" t="n"/>
+      <c r="K87" s="39" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="B88" s="39" t="inlineStr">
@@ -1695,6 +1705,11 @@
         </is>
       </c>
       <c r="J88" s="17" t="n"/>
+      <c r="K88" s="39" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="J89" s="17" t="n"/>
@@ -1714,6 +1729,11 @@
         </is>
       </c>
       <c r="J91" s="17" t="n"/>
+      <c r="K91" s="39" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="J92" s="17" t="n"/>
@@ -1733,6 +1753,11 @@
         </is>
       </c>
       <c r="J94" s="17" t="n"/>
+      <c r="K94" s="39" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="B95" s="39" t="inlineStr">
@@ -1741,6 +1766,11 @@
         </is>
       </c>
       <c r="J95" s="17" t="n"/>
+      <c r="K95" s="39" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="J96" s="17" t="n"/>
@@ -1760,6 +1790,11 @@
         </is>
       </c>
       <c r="J98" s="17" t="n"/>
+      <c r="K98" s="39" t="inlineStr">
+        <is>
+          <t>FIXED - Added individual/test email input with chips and multi-recipient support in broadcast modals and backend API.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="B99" s="39" t="inlineStr">
@@ -1768,6 +1803,11 @@
         </is>
       </c>
       <c r="J99" s="17" t="n"/>
+      <c r="K99" s="39" t="inlineStr">
+        <is>
+          <t>FIXED - Resolved Zoho SMTP relay and port configuration; verified email delivery in production.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="J100" s="17" t="n"/>
@@ -1787,6 +1827,11 @@
         </is>
       </c>
       <c r="J102" s="17" t="n"/>
+      <c r="K102" s="39" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="B103" s="39" t="inlineStr">
@@ -1795,6 +1840,11 @@
         </is>
       </c>
       <c r="J103" s="17" t="n"/>
+      <c r="K103" s="39" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="J104" s="17" t="n"/>
@@ -1814,6 +1864,11 @@
         </is>
       </c>
       <c r="J106" s="17" t="n"/>
+      <c r="K106" s="39" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="B107" s="39" t="inlineStr">
@@ -1822,6 +1877,11 @@
         </is>
       </c>
       <c r="J107" s="17" t="n"/>
+      <c r="K107" s="39" t="inlineStr">
+        <is>
+          <t>Pending Implementation</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="J108" s="17" t="n"/>

</xml_diff>

<commit_message>
feat(global): enhance Important Updates and Placements with Sr No, candidate link, sorting, and uniform dates
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -1589,7 +1589,7 @@
       </c>
       <c r="K79" s="36" t="inlineStr">
         <is>
-          <t>Pending Implementation</t>
+          <t>FIXED - Added formatName helper capitalizing 1st letter of names across tables and profiles.</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="K80" s="36" t="inlineStr">
         <is>
-          <t>Pending Implementation</t>
+          <t>FIXED - Made Candidate Name clickable linking directly to Candidate Profile on Important Updates and Placements.</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="K81" s="36" t="inlineStr">
         <is>
-          <t>Pending Implementation</t>
+          <t>FIXED - Added column sorting with indicators for Status, Interview Date, ETS Date, Applied, Candidate, and Job.</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="K82" s="36" t="inlineStr">
         <is>
-          <t>Pending Implementation</t>
+          <t>FIXED - Standardized date formatting globally to uniform 26-Oct-2026 (DD-MMM-YYYY) in fmtDate.</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="K83" s="36" t="inlineStr">
         <is>
-          <t>Pending Implementation</t>
+          <t>FIXED - Removed non-functional AI Screen button from Important Updates pipeline and list views.</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       <c r="J86" s="17" t="n"/>
       <c r="K86" s="39" t="inlineStr">
         <is>
-          <t>Pending Implementation</t>
+          <t>FIXED - Added sequential Sr No (#) and Candidate ID (JS-XXX) next to candidate names in Placements.</t>
         </is>
       </c>
     </row>
@@ -1694,7 +1694,7 @@
       <c r="J87" s="17" t="n"/>
       <c r="K87" s="39" t="inlineStr">
         <is>
-          <t>Pending Implementation</t>
+          <t>FIXED - Made Candidate Name in Placements clickable redirecting directly to Candidate Profile.</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1707,7 @@
       <c r="J88" s="17" t="n"/>
       <c r="K88" s="39" t="inlineStr">
         <is>
-          <t>Pending Implementation</t>
+          <t>FIXED - Added column sorting on Placements table (Candidate, Job, Employer, Provider, Start Date, Wage Sub Status).</t>
         </is>
       </c>
     </row>
@@ -1866,7 +1866,7 @@
       <c r="J106" s="17" t="n"/>
       <c r="K106" s="39" t="inlineStr">
         <is>
-          <t>Pending Implementation</t>
+          <t>FIXED - Added candidate_sr_no (JS-XXX) in API and displayed on Important Updates and Placements.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: format CRM improvements spreadsheet and update all completed statuses
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -13,7 +13,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -93,6 +93,11 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00166534"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -152,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -229,6 +234,9 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -507,9 +515,17 @@
   <dimension ref="A1:X1017"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="15" customWidth="1" style="29" min="4" max="4"/>
-    <col width="15.25" customWidth="1" style="29" min="7" max="8"/>
-    <col width="129.13" customWidth="1" style="29" min="10" max="10"/>
+    <col width="25" customWidth="1" style="29" min="1" max="1"/>
+    <col width="50" customWidth="1" style="29" min="2" max="2"/>
+    <col width="3" customWidth="1" style="29" min="3" max="3"/>
+    <col width="3" customWidth="1" style="29" min="4" max="4"/>
+    <col width="3" customWidth="1" style="29" min="5" max="5"/>
+    <col width="3" customWidth="1" style="29" min="6" max="6"/>
+    <col width="3" customWidth="1" style="29" min="7" max="8"/>
+    <col width="3" customWidth="1" style="29" min="8" max="8"/>
+    <col width="3" customWidth="1" style="29" min="9" max="9"/>
+    <col width="12" customWidth="1" style="29" min="10" max="10"/>
+    <col width="65" customWidth="1" style="29" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1565,14 +1581,10 @@
           <t>1. Add Sr No to Candidate Names (first column) easy referencing during meeting... 1,2,3,4,5... (On All Tabs Candidates, Important Updates, Providers, Traning Program etc)</t>
         </is>
       </c>
-      <c r="J78" s="35" t="inlineStr">
-        <is>
-          <t>Add sequential row numbers (# / Sr No) in the first column across all primary data tables (Candidates, Important Updates, Providers, Training Program, etc.) for easy referencing during team meetings.</t>
-        </is>
-      </c>
-      <c r="K78" s="36" t="inlineStr">
-        <is>
-          <t>Pending Implementation</t>
+      <c r="J78" s="35" t="n"/>
+      <c r="K78" s="40" t="inlineStr">
+        <is>
+          <t>FIXED - Added Candidate SR # (JS-XXX) pill badge across all primary pages: Candidates, Important Updates, Placements, Training Enrolments, Job Detail, Dashboard, Reports, Placement Detail, Employer Detail, Provider Detail, and modals.</t>
         </is>
       </c>
     </row>
@@ -1582,12 +1594,8 @@
           <t>2. Coding required for better formatting and uniformity so the 1st Letter in First Name and Last Name is Capital (Kavil Desai)</t>
         </is>
       </c>
-      <c r="J79" s="35" t="inlineStr">
-        <is>
-          <t>Enforce title case / proper capitalization (First letter of First and Last Name capitalized) across all names and input fields (Candidate Name, Vacancies, Employers, Providers, Consultants, Training Program).</t>
-        </is>
-      </c>
-      <c r="K79" s="36" t="inlineStr">
+      <c r="J79" s="35" t="n"/>
+      <c r="K79" s="40" t="inlineStr">
         <is>
           <t>FIXED - Added formatName helper capitalizing 1st letter of names across tables and profiles.</t>
         </is>
@@ -1599,12 +1607,8 @@
           <t>3. Can the Important Updates or anywhere the Candidate Name appears can have a link which can redirect to Candidate Profile directly for quick edits</t>
         </is>
       </c>
-      <c r="J80" s="37" t="inlineStr">
-        <is>
-          <t>Make Candidate Names clickable links in Important Updates and application tables redirecting directly to Candidate Profile for quick viewing and edits.</t>
-        </is>
-      </c>
-      <c r="K80" s="36" t="inlineStr">
+      <c r="J80" s="37" t="n"/>
+      <c r="K80" s="40" t="inlineStr">
         <is>
           <t>FIXED - Made Candidate Name clickable linking directly to Candidate Profile on Important Updates and Placements.</t>
         </is>
@@ -1616,12 +1620,8 @@
           <t>4. Sorting Feature for Status , Interview Dates, ETS, Applies etc... so we can view all that we want to see quicker</t>
         </is>
       </c>
-      <c r="J81" s="37" t="inlineStr">
-        <is>
-          <t>Add interactive column sorting (Status, Interview Date, ETS Date, Applied Date) in Important Updates and pipeline tables.</t>
-        </is>
-      </c>
-      <c r="K81" s="36" t="inlineStr">
+      <c r="J81" s="37" t="n"/>
+      <c r="K81" s="40" t="inlineStr">
         <is>
           <t>FIXED - Added column sorting with indicators for Status, Interview Date, ETS Date, Applied, Candidate, and Job.</t>
         </is>
@@ -1633,12 +1633,8 @@
           <t>5. Date Formatting : Can we have uniform date format everywhere as 26-Oct-2026</t>
         </is>
       </c>
-      <c r="J82" s="37" t="inlineStr">
-        <is>
-          <t>Standardize date display format everywhere across the entire application to uniform DD-MMM-YYYY (e.g. 26-Oct-2026).</t>
-        </is>
-      </c>
-      <c r="K82" s="36" t="inlineStr">
+      <c r="J82" s="37" t="n"/>
+      <c r="K82" s="40" t="inlineStr">
         <is>
           <t>FIXED - Standardized date formatting globally to uniform 26-Oct-2026 (DD-MMM-YYYY) in fmtDate.</t>
         </is>
@@ -1650,12 +1646,8 @@
           <t>6. Ai Screen: If this feature is non functional, please remove it</t>
         </is>
       </c>
-      <c r="J83" s="37" t="inlineStr">
-        <is>
-          <t>Remove non-functional AI Screen button from the Important Updates action column.</t>
-        </is>
-      </c>
-      <c r="K83" s="36" t="inlineStr">
+      <c r="J83" s="37" t="n"/>
+      <c r="K83" s="40" t="inlineStr">
         <is>
           <t>FIXED - Removed non-functional AI Screen button from Important Updates pipeline and list views.</t>
         </is>
@@ -1665,7 +1657,7 @@
       <c r="J84" s="17" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="38" t="inlineStr">
+      <c r="A85" s="34" t="inlineStr">
         <is>
           <t>Placements</t>
         </is>
@@ -1673,39 +1665,39 @@
       <c r="J85" s="17" t="n"/>
     </row>
     <row r="86">
-      <c r="B86" s="39" t="inlineStr">
+      <c r="B86" s="35" t="inlineStr">
         <is>
           <t>1. SR No on the side of Candidate Name</t>
         </is>
       </c>
       <c r="J86" s="17" t="n"/>
-      <c r="K86" s="39" t="inlineStr">
+      <c r="K86" s="40" t="inlineStr">
         <is>
           <t>FIXED - Added sequential Sr No (#) and Candidate ID (JS-XXX) next to candidate names in Placements.</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="B87" s="39" t="inlineStr">
+      <c r="B87" s="35" t="inlineStr">
         <is>
           <t>2. Candidate Name clickable to Candidate Profile</t>
         </is>
       </c>
       <c r="J87" s="17" t="n"/>
-      <c r="K87" s="39" t="inlineStr">
+      <c r="K87" s="40" t="inlineStr">
         <is>
           <t>FIXED - Made Candidate Name in Placements clickable redirecting directly to Candidate Profile.</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="B88" s="39" t="inlineStr">
+      <c r="B88" s="35" t="inlineStr">
         <is>
           <t>3. Sorting Feature</t>
         </is>
       </c>
       <c r="J88" s="17" t="n"/>
-      <c r="K88" s="39" t="inlineStr">
+      <c r="K88" s="40" t="inlineStr">
         <is>
           <t>FIXED - Added column sorting on Placements table (Candidate, Job, Employer, Provider, Start Date, Wage Sub Status).</t>
         </is>
@@ -1715,7 +1707,7 @@
       <c r="J89" s="17" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="38" t="inlineStr">
+      <c r="A90" s="34" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
@@ -1723,13 +1715,13 @@
       <c r="J90" s="17" t="n"/>
     </row>
     <row r="91">
-      <c r="B91" s="39" t="inlineStr">
+      <c r="B91" s="35" t="inlineStr">
         <is>
           <t>1. ETS information Mismatch (align top summary card "ETS This Month" with Hiring Pipeline "ETS" stage distribution)</t>
         </is>
       </c>
       <c r="J91" s="17" t="n"/>
-      <c r="K91" s="39" t="inlineStr">
+      <c r="K91" s="40" t="inlineStr">
         <is>
           <t>FIXED - Added ets stage to by_stage in stats API and aligned dashboard ETS metric with Hiring Pipeline funnel.</t>
         </is>
@@ -1739,7 +1731,7 @@
       <c r="J92" s="17" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="38" t="inlineStr">
+      <c r="A93" s="34" t="inlineStr">
         <is>
           <t>Employers</t>
         </is>
@@ -1747,28 +1739,28 @@
       <c r="J93" s="17" t="n"/>
     </row>
     <row r="94">
-      <c r="B94" s="39" t="inlineStr">
+      <c r="B94" s="35" t="inlineStr">
         <is>
           <t>1. Sr No next to Company Name</t>
         </is>
       </c>
       <c r="J94" s="17" t="n"/>
-      <c r="K94" s="39" t="inlineStr">
-        <is>
-          <t>Pending Implementation</t>
+      <c r="K94" s="40" t="inlineStr">
+        <is>
+          <t>FIXED - Added sequential SR # column next to Company Name in Employers table for quick meeting referencing.</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="B95" s="39" t="inlineStr">
+      <c r="B95" s="35" t="inlineStr">
         <is>
           <t>2. Deactivate and Delete Option required (maybe delete option in the company profile menu inside)</t>
         </is>
       </c>
       <c r="J95" s="17" t="n"/>
-      <c r="K95" s="39" t="inlineStr">
-        <is>
-          <t>Pending Implementation</t>
+      <c r="K95" s="40" t="inlineStr">
+        <is>
+          <t>FIXED - Added active/inactive toggle switch directly in the Employers list and permanent Delete option with confirmation modal and single-row layout.</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1768,7 @@
       <c r="J96" s="17" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="38" t="inlineStr">
+      <c r="A97" s="34" t="inlineStr">
         <is>
           <t>Broadcast Email</t>
         </is>
@@ -1784,26 +1776,26 @@
       <c r="J97" s="17" t="n"/>
     </row>
     <row r="98">
-      <c r="B98" s="39" t="inlineStr">
+      <c r="B98" s="35" t="inlineStr">
         <is>
           <t>1. Add individual email option in Broadcast Selected Vacancies modal</t>
         </is>
       </c>
       <c r="J98" s="17" t="n"/>
-      <c r="K98" s="39" t="inlineStr">
+      <c r="K98" s="40" t="inlineStr">
         <is>
           <t>FIXED - Added individual/test email input with chips and multi-recipient support in broadcast modals and backend API.</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="B99" s="39" t="inlineStr">
+      <c r="B99" s="35" t="inlineStr">
         <is>
           <t>2. Broadcast Email delivery check: Verify email delivery when tested with WV Employer profile (e.g. sent to dhaval@workvision.com.au)</t>
         </is>
       </c>
       <c r="J99" s="17" t="n"/>
-      <c r="K99" s="39" t="inlineStr">
+      <c r="K99" s="40" t="inlineStr">
         <is>
           <t>FIXED - Resolved Zoho SMTP relay and port configuration; verified email delivery in production.</t>
         </is>
@@ -1813,7 +1805,7 @@
       <c r="J100" s="17" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="38" t="inlineStr">
+      <c r="A101" s="34" t="inlineStr">
         <is>
           <t>Candidate Assignment &amp; Staff KPI</t>
         </is>
@@ -1821,28 +1813,28 @@
       <c r="J101" s="17" t="n"/>
     </row>
     <row r="102">
-      <c r="B102" s="39" t="inlineStr">
+      <c r="B102" s="35" t="inlineStr">
         <is>
           <t>1. Managed By .. Staff Name .. Drop Down List on Candidate Profile to know who is working with the candidate</t>
         </is>
       </c>
       <c r="J102" s="17" t="n"/>
-      <c r="K102" s="39" t="inlineStr">
-        <is>
-          <t>Pending Implementation</t>
+      <c r="K102" s="40" t="inlineStr">
+        <is>
+          <t>FIXED - Added staff_id to database &amp; candidate model; added Managed By staff dropdown selector in Communication Notes header and edit view with safe backfill from created_by.</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="B103" s="39" t="inlineStr">
+      <c r="B103" s="35" t="inlineStr">
         <is>
           <t>2. Reflect assigned staff member in Reports under Staff KPI and Placements</t>
         </is>
       </c>
       <c r="J103" s="17" t="n"/>
-      <c r="K103" s="39" t="inlineStr">
-        <is>
-          <t>Pending Implementation</t>
+      <c r="K103" s="40" t="inlineStr">
+        <is>
+          <t>FIXED - Added Managed By column in Placement Report Month Wise table and CSV export; added Managed Candidates count and placement attribution to Staff KPI Placement Report and CSV export.</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1842,7 @@
       <c r="J104" s="17" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="38" t="inlineStr">
+      <c r="A105" s="34" t="inlineStr">
         <is>
           <t>Candidates Tab &amp; Global Candidate ID</t>
         </is>
@@ -1858,26 +1850,26 @@
       <c r="J105" s="17" t="n"/>
     </row>
     <row r="106">
-      <c r="B106" s="39" t="inlineStr">
+      <c r="B106" s="35" t="inlineStr">
         <is>
           <t>1. Consistent Candidate SR No. (e.g. JS-046) across all other pages once assigned to a candidate</t>
         </is>
       </c>
       <c r="J106" s="17" t="n"/>
-      <c r="K106" s="39" t="inlineStr">
+      <c r="K106" s="40" t="inlineStr">
         <is>
           <t>FIXED - Candidate SR # (JS-XXX) pill badge implemented across all pages: Important Updates, Placements, Training Enrolments, Job Detail, Dashboard, Reports, Placement Detail, Employer Detail, Provider Detail, and modals.</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="B107" s="39" t="inlineStr">
+      <c r="B107" s="35" t="inlineStr">
         <is>
           <t>2. Freeze First Column in Candidate Tab when scrolled horizontally so candidate name remains visible while updating dates etc.</t>
         </is>
       </c>
       <c r="J107" s="17" t="n"/>
-      <c r="K107" s="39" t="inlineStr">
+      <c r="K107" s="40" t="inlineStr">
         <is>
           <t>FIXED - Frozen SR # and Candidate Name columns on horizontal scroll with sticky headers and cells.</t>
         </is>

</xml_diff>

<commit_message>
docs: update CRM Improvements spreadsheet with Training Program formatting enhancements
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -1224,7 +1224,21 @@
       </c>
     </row>
     <row r="54">
-      <c r="J54" s="17" t="n"/>
+      <c r="B54" s="35" t="inlineStr">
+        <is>
+          <t>Format Training Program table width and prevent multi-line wrapping</t>
+        </is>
+      </c>
+      <c r="J54" s="37" t="inlineStr">
+        <is>
+          <t>Expanded container width and enforced whitespace-nowrap across candidate, course, dates, and actions.</t>
+        </is>
+      </c>
+      <c r="K54" s="40" t="inlineStr">
+        <is>
+          <t>COMPLETED - Expanded container width, removed flex-wrap, and prevented multi-line wrapping on candidate, course, dates, and actions.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="22" t="inlineStr">
@@ -1879,10 +1893,25 @@
       <c r="J108" s="17" t="n"/>
     </row>
     <row r="109">
+      <c r="A109" s="34" t="inlineStr">
+        <is>
+          <t>Training Program</t>
+        </is>
+      </c>
       <c r="J109" s="17" t="n"/>
     </row>
     <row r="110">
+      <c r="B110" s="35" t="inlineStr">
+        <is>
+          <t>1. Format Training Program: Increase width, prevent candidate name, course title, dates, and edit/open buttons from wrapping onto two lines</t>
+        </is>
+      </c>
       <c r="J110" s="17" t="n"/>
+      <c r="K110" s="40" t="inlineStr">
+        <is>
+          <t>FIXED - Expanded container width (up to 1600px), removed flex-wrap, enforced whitespace-nowrap and column min-widths for Candidate, Course, Dates, Cert Received, and inline Edit · Open action buttons, with responsive horizontal scroll.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="J111" s="17" t="n"/>

</xml_diff>

<commit_message>
docs: add clear column headers to CRM Improvements spreadsheet
</commit_message>
<xml_diff>
--- a/doc/CRM Improvements .xlsx
+++ b/doc/CRM Improvements .xlsx
@@ -157,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -236,6 +236,12 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -529,8 +535,16 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="n"/>
-      <c r="B1" s="2" t="n"/>
+      <c r="A1" s="41" t="inlineStr">
+        <is>
+          <t>Module / Category</t>
+        </is>
+      </c>
+      <c r="B1" s="41" t="inlineStr">
+        <is>
+          <t>Enhancement / Requirement</t>
+        </is>
+      </c>
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="3" t="n"/>
       <c r="E1" s="3" t="n"/>
@@ -538,12 +552,12 @@
       <c r="G1" s="3" t="n"/>
       <c r="H1" s="3" t="n"/>
       <c r="I1" s="3" t="n"/>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>Comment</t>
-        </is>
-      </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="J1" s="42" t="inlineStr">
+        <is>
+          <t>Comment / Details</t>
+        </is>
+      </c>
+      <c r="K1" s="41" t="inlineStr">
         <is>
           <t>Status</t>
         </is>

</xml_diff>